<commit_message>
Add initial company list CSV file with 373 entries
</commit_message>
<xml_diff>
--- a/NEPSE_Trading_Reports/NEPSE_Company_Summary.xlsx
+++ b/NEPSE_Trading_Reports/NEPSE_Company_Summary.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>126765.37</v>
+        <v>5258.55</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>219</v>
+        <v>11</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>219</v>
+        <v>11</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>153042.7</v>
+        <v>11832.37</v>
       </c>
     </row>
     <row r="6">
@@ -545,358 +545,2790 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>179778.67</v>
+        <v>3819.18</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>474</v>
+        <v>12</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>474</v>
+        <v>12</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>249080.46</v>
+        <v>9240.120000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>BBC</t>
+          <t>ALBSL</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>988829</v>
+        <v>17209.2</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1323098.47</v>
+        <v>17210.12</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CHCL</t>
+          <t>ALICL</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>137945.13</v>
+        <v>8228.65</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>238</v>
+        <v>11</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>238</v>
+        <v>11</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>169084.12</v>
+        <v>8939.26</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CIT</t>
+          <t>ANLB</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>205896.49</v>
+        <v>520600.61</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>225420.74</v>
+        <v>645345</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>CZBIL</t>
+          <t>AVYAN</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>184027.66</v>
+        <v>9347.83</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>618</v>
+        <v>12</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>618</v>
+        <v>12</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>214932.19</v>
+        <v>16301.94</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>EBL</t>
+          <t>BANDIPUR</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>397779.14</v>
+        <v>11417.56</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>416</v>
+        <v>10</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>416</v>
+        <v>10</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>466424.75</v>
+        <v>11332.25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>GBIME</t>
+          <t>BBC</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>103919.7</v>
+        <v>360621.73</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>297</v>
+        <v>70</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>297</v>
+        <v>70</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>125119.74</v>
+        <v>484576.95</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>HDL</t>
+          <t>BEDC</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>789262.5600000001</v>
+        <v>9785.469999999999</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>315</v>
+        <v>11</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>315</v>
+        <v>11</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1310668.82</v>
+        <v>10363.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>KBL</t>
+          <t>BHCL</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>229051.75</v>
+        <v>29483.17</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>1015</v>
+        <v>55</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1015</v>
+        <v>55</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>257260.14</v>
+        <v>36582.01</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>LICN</t>
+          <t>BHPL</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>521500.81</v>
+        <v>11397.49</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>282</v>
+        <v>10</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>282</v>
+        <v>10</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>590872.26</v>
+        <v>12378.31</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>NABIL</t>
+          <t>BNHC</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>263290.78</v>
+        <v>6212.12</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>199</v>
+        <v>10</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>199</v>
+        <v>10</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>277942.18</v>
+        <v>7387.1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>NFS</t>
+          <t>BNT</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>226850.96</v>
+        <v>1043743.76</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>419</v>
+        <v>70</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>419</v>
+        <v>70</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>822920.8100000001</v>
+        <v>1177901.59</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>NIMB</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>19748.08</v>
+        <v>9303.18</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>91</v>
+        <v>11</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>91</v>
+        <v>11</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>21947.43</v>
+        <v>11298.46</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>NLIC</t>
+          <t>CBLD88</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>396786</v>
+        <v>12421.31</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>226</v>
+        <v>10</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>226</v>
+        <v>10</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>433113.44</v>
+        <v>13195.24</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>NTC</t>
+          <t>CHDC</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>526131.01</v>
+        <v>163583.39</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>560</v>
+        <v>70</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>560</v>
+        <v>70</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>878852.45</v>
+        <v>202494.73</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>SCB</t>
+          <t>CHL</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>311933.96</v>
+        <v>13029.49</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>410</v>
+        <v>39</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>410</v>
+        <v>39</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>399358.31</v>
+        <v>24363.11</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>SHPC</t>
+          <t>CORBL</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>290980.81</v>
+        <v>75710.17999999999</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>576</v>
+        <v>40</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>576</v>
+        <v>40</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>380092.35</v>
+        <v>110204.8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>STC</t>
+          <t>CREST</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>2588730.52</v>
+        <v>31547.87</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>470</v>
+        <v>20</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>470</v>
+        <v>20</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>3015330.37</v>
+        <v>34325.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>TPC</t>
+          <t>CYCL</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>477861.72</v>
+        <v>166648.95</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>1026</v>
+        <v>70</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>1026</v>
+        <v>70</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>575496.23</v>
+        <v>182796.3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>DDBL</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>10524.23</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>11282.44</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>DHPL</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>4452.54</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>4808.9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>DLBS</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>53589.64</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>132942.13</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>EBL</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>55738.05</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>75565.38</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>EHPL</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>28093.88</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>30213.98</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>ENL</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>83343.12</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>92</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>92</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>133835.5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>GBBL</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>65949.73</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>163</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>163</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>116744.9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>GBLBS</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>12873</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>13783.02</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>GFCL</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>17157.91</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>37050.35</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>GILB</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>85343.38</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>148316.25</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>GLBSL</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>206837.09</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>232281</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>GMFBS</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>20852.81</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>22709.42</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>GMLI</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>161387.71</v>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>237221.01</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>GRDBL</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>62018.32</v>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>71847.28</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>GUFL</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>46604.65</v>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>57142.73</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>GVL</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>19523.76</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>38116.04</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>HDL</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>281335.41</v>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>547256.4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>HIMSTAR</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>48104.85</v>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>95536.91</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>HURJA</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>9636.91</v>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>9897.65</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>ICFCD88</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>22358.34</v>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D44" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>24178.8</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ILBS</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>12334.79</v>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>12598.68</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>JBLB</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>526497.79</v>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>130</v>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>130</v>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>630908.99</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>JSLBB</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>133106.73</v>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>286760.05</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>KBLD90</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>15031.06</v>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E48" s="5" t="n">
+        <v>14918.75</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>KBSH</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>234526.34</v>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>295661.25</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>4946.38</v>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>495</v>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>495</v>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>5453.48</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>KMCDB</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>60851.87</v>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E51" s="5" t="n">
+        <v>124256.81</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>LICN</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>129925.85</v>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="D52" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>145201.88</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>LLBS</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>24707.21</v>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E53" s="5" t="n">
+        <v>25120.35</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>LUK</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10990.3</v>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>1098</v>
+      </c>
+      <c r="D54" s="6" t="n">
+        <v>1098</v>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v>12868.75</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>MABEL</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>48858.77</v>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="E55" s="5" t="n">
+        <v>74800.96000000001</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>MBJC</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>61791.69</v>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="D56" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="E56" s="5" t="n">
+        <v>84978.48</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>73236.96000000001</v>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>106</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>106</v>
+      </c>
+      <c r="E57" s="5" t="n">
+        <v>136791.44</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>MEGA</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>12196.37</v>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v>13128.4</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>MERO</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n">
+        <v>15493.79</v>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E59" s="5" t="n">
+        <v>16862.43</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>MFIL</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="n">
+        <v>17999.06</v>
+      </c>
+      <c r="C60" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="D60" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="E60" s="5" t="n">
+        <v>23461.5</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>MHNL</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n">
+        <v>6697.93</v>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E61" s="5" t="n">
+        <v>8164.18</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>MLBBL</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="n">
+        <v>64144.36</v>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E62" s="5" t="n">
+        <v>68865.5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>MLBL</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>6704.96</v>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E63" s="5" t="n">
+        <v>9640.620000000001</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>MLBLD89</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="n">
+        <v>12571.88</v>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D64" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E64" s="5" t="n">
+        <v>13424.38</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>MLBS</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>44356.63</v>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="E65" s="5" t="n">
+        <v>79625</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>MLBSL</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n">
+        <v>324587.01</v>
+      </c>
+      <c r="C66" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="D66" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="E66" s="5" t="n">
+        <v>364572.05</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>MPFL</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>9811.559999999999</v>
+      </c>
+      <c r="C67" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E67" s="5" t="n">
+        <v>44208.5</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>NABBC</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="n">
+        <v>108002.75</v>
+      </c>
+      <c r="C68" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="D68" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="E68" s="5" t="n">
+        <v>154761.52</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>NBF2</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="n">
+        <v>10190.22</v>
+      </c>
+      <c r="C69" s="6" t="n">
+        <v>976</v>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>976</v>
+      </c>
+      <c r="E69" s="5" t="n">
+        <v>11295.2</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>NBLD85</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="n">
+        <v>10745.05</v>
+      </c>
+      <c r="C70" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D70" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E70" s="5" t="n">
+        <v>11800.49</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>NESDO</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="n">
+        <v>283839.3</v>
+      </c>
+      <c r="C71" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="E71" s="5" t="n">
+        <v>431873.28</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>NFS</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="n">
+        <v>61574.76</v>
+      </c>
+      <c r="C72" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D72" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E72" s="5" t="n">
+        <v>71017.41</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>NGPL</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="n">
+        <v>20437.17</v>
+      </c>
+      <c r="C73" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="E73" s="5" t="n">
+        <v>28068.16</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>NHPC</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="n">
+        <v>2554.45</v>
+      </c>
+      <c r="C74" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D74" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E74" s="5" t="n">
+        <v>6920.85</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>NICA</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="n">
+        <v>9347.83</v>
+      </c>
+      <c r="C75" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E75" s="5" t="n">
+        <v>10076.98</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>NICBF</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="n">
+        <v>209.69</v>
+      </c>
+      <c r="C76" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D76" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E76" s="5" t="n">
+        <v>159.59</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>NICL</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="n">
+        <v>23527.72</v>
+      </c>
+      <c r="C77" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E77" s="5" t="n">
+        <v>29399.15</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>NICSF</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="n">
+        <v>9990.4</v>
+      </c>
+      <c r="C78" s="6" t="n">
+        <v>1071</v>
+      </c>
+      <c r="D78" s="6" t="n">
+        <v>1071</v>
+      </c>
+      <c r="E78" s="5" t="n">
+        <v>12031.92</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>NIL</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="n">
+        <v>11738.76</v>
+      </c>
+      <c r="C79" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E79" s="5" t="n">
+        <v>18196.41</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>NLG</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="n">
+        <v>12722.44</v>
+      </c>
+      <c r="C80" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E80" s="5" t="n">
+        <v>13673.44</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>NLIC</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="n">
+        <v>185119.33</v>
+      </c>
+      <c r="C81" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="E81" s="5" t="n">
+        <v>205421.3</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>NMB</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="n">
+        <v>2583.56</v>
+      </c>
+      <c r="C82" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D82" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E82" s="5" t="n">
+        <v>2687.79</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>NMB50</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="n">
+        <v>1386.69</v>
+      </c>
+      <c r="C83" s="6" t="n">
+        <v>102</v>
+      </c>
+      <c r="D83" s="6" t="n">
+        <v>102</v>
+      </c>
+      <c r="E83" s="5" t="n">
+        <v>1773.63</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>NMBMF</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>86131.60000000001</v>
+      </c>
+      <c r="C84" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E84" s="5" t="n">
+        <v>90519.08</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>NMFBS</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="n">
+        <v>34855.12</v>
+      </c>
+      <c r="C85" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D85" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E85" s="5" t="n">
+        <v>36437.75</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>NMIC</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="n">
+        <v>166575.49</v>
+      </c>
+      <c r="C86" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="D86" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E86" s="5" t="n">
+        <v>237291.46</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>NRIC</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="n">
+        <v>16945.41</v>
+      </c>
+      <c r="C87" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D87" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E87" s="5" t="n">
+        <v>17228.95</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>NRN</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="n">
+        <v>151201.94</v>
+      </c>
+      <c r="C88" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="D88" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="E88" s="5" t="n">
+        <v>190758</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>NTC</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="n">
+        <v>22895.35</v>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="E89" s="5" t="n">
+        <v>42485.89</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>NUBL</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="n">
+        <v>22649.53</v>
+      </c>
+      <c r="C90" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D90" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E90" s="5" t="n">
+        <v>24831.44</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>NYADI</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="n">
+        <v>9829.629999999999</v>
+      </c>
+      <c r="C91" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D91" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E91" s="5" t="n">
+        <v>10351.94</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>OHL</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="n">
+        <v>15584.03</v>
+      </c>
+      <c r="C92" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D92" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E92" s="5" t="n">
+        <v>35513.14</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>OMPL</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="n">
+        <v>130326.66</v>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>114</v>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>114</v>
+      </c>
+      <c r="E93" s="5" t="n">
+        <v>221976.03</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>PBLD84</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="n">
+        <v>10918.7</v>
+      </c>
+      <c r="C94" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D94" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E94" s="5" t="n">
+        <v>11515.56</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>PFL</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="n">
+        <v>9811.559999999999</v>
+      </c>
+      <c r="C95" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D95" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E95" s="5" t="n">
+        <v>12916.29</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>PHCL</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="n">
+        <v>19322.4</v>
+      </c>
+      <c r="C96" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="D96" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="E96" s="5" t="n">
+        <v>24462.53</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>PLIC</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="n">
+        <v>23091.17</v>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D97" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E97" s="5" t="n">
+        <v>28816.44</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>PMHPL</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="n">
+        <v>19604.73</v>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="D98" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="E98" s="5" t="n">
+        <v>20986.04</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>PROFL</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="n">
+        <v>13963.89</v>
+      </c>
+      <c r="C99" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="D99" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="E99" s="5" t="n">
+        <v>47059.68</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>PSF</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="n">
+        <v>1547.88</v>
+      </c>
+      <c r="C100" s="6" t="n">
+        <v>162</v>
+      </c>
+      <c r="D100" s="6" t="n">
+        <v>162</v>
+      </c>
+      <c r="E100" s="5" t="n">
+        <v>1948.87</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>PURE</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="n">
+        <v>112621.63</v>
+      </c>
+      <c r="C101" s="6" t="n">
+        <v>133</v>
+      </c>
+      <c r="D101" s="6" t="n">
+        <v>133</v>
+      </c>
+      <c r="E101" s="5" t="n">
+        <v>161376.52</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>RADHI</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="n">
+        <v>31318.72</v>
+      </c>
+      <c r="C102" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D102" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="E102" s="5" t="n">
+        <v>39276.88</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>RAWA</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="n">
+        <v>9540.549999999999</v>
+      </c>
+      <c r="C103" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D103" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E103" s="5" t="n">
+        <v>11523.53</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>RBCL</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="n">
+        <v>2267330.21</v>
+      </c>
+      <c r="C104" s="6" t="n">
+        <v>140</v>
+      </c>
+      <c r="D104" s="6" t="n">
+        <v>140</v>
+      </c>
+      <c r="E104" s="5" t="n">
+        <v>2502325.82</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>RBCLPO</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="n">
+        <v>1123873.05</v>
+      </c>
+      <c r="C105" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="D105" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E105" s="5" t="n">
+        <v>1213895.47</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>RFPL</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="n">
+        <v>20837.66</v>
+      </c>
+      <c r="C106" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D106" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E106" s="5" t="n">
+        <v>29518.7</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>RIDI</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="n">
+        <v>9932.01</v>
+      </c>
+      <c r="C107" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D107" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E107" s="5" t="n">
+        <v>11511.58</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>RRHP</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="n">
+        <v>19579.96</v>
+      </c>
+      <c r="C108" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="D108" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E108" s="5" t="n">
+        <v>19884.96</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>RSML</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="n">
+        <v>106744.32</v>
+      </c>
+      <c r="C109" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D109" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E109" s="5" t="n">
+        <v>238925.2</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>SABBL</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="n">
+        <v>103340.02</v>
+      </c>
+      <c r="C110" s="6" t="n">
+        <v>107</v>
+      </c>
+      <c r="D110" s="6" t="n">
+        <v>107</v>
+      </c>
+      <c r="E110" s="5" t="n">
+        <v>196780.17</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>SADBL</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="n">
+        <v>5434.21</v>
+      </c>
+      <c r="C111" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D111" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="E111" s="5" t="n">
+        <v>10052.07</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>SAGAR</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="n">
+        <v>178220.11</v>
+      </c>
+      <c r="C112" s="6" t="n">
+        <v>124</v>
+      </c>
+      <c r="D112" s="6" t="n">
+        <v>124</v>
+      </c>
+      <c r="E112" s="5" t="n">
+        <v>291242.6</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>SANIMA</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="n">
+        <v>9546.57</v>
+      </c>
+      <c r="C113" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D113" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="E113" s="5" t="n">
+        <v>15708.78</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>SAPDBL</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="n">
+        <v>26149.51</v>
+      </c>
+      <c r="C114" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D114" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E114" s="5" t="n">
+        <v>26804.42</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>SBCF</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="n">
+        <v>15897.01</v>
+      </c>
+      <c r="C115" s="6" t="n">
+        <v>1611</v>
+      </c>
+      <c r="D115" s="6" t="n">
+        <v>1611</v>
+      </c>
+      <c r="E115" s="5" t="n">
+        <v>18390.97</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>SBI</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="n">
+        <v>29672.68</v>
+      </c>
+      <c r="C116" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="D116" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="E116" s="5" t="n">
+        <v>43750.04</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>SBL</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="n">
+        <v>14228.06</v>
+      </c>
+      <c r="C117" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D117" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E117" s="5" t="n">
+        <v>14081.9</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>SBLD89</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="n">
+        <v>28054.63</v>
+      </c>
+      <c r="C118" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D118" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E118" s="5" t="n">
+        <v>29837.5</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>SEF</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="n">
+        <v>9997.51</v>
+      </c>
+      <c r="C119" s="6" t="n">
+        <v>975</v>
+      </c>
+      <c r="D119" s="6" t="n">
+        <v>975</v>
+      </c>
+      <c r="E119" s="5" t="n">
+        <v>11184.31</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>SFCL</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="n">
+        <v>9580.700000000001</v>
+      </c>
+      <c r="C120" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D120" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="E120" s="5" t="n">
+        <v>17187.31</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>SFEF</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="n">
+        <v>9989.950000000001</v>
+      </c>
+      <c r="C121" s="6" t="n">
+        <v>981</v>
+      </c>
+      <c r="D121" s="6" t="n">
+        <v>981</v>
+      </c>
+      <c r="E121" s="5" t="n">
+        <v>10334.61</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>SFMF</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="n">
+        <v>9989.360000000001</v>
+      </c>
+      <c r="C122" s="6" t="n">
+        <v>961</v>
+      </c>
+      <c r="D122" s="6" t="n">
+        <v>961</v>
+      </c>
+      <c r="E122" s="5" t="n">
+        <v>10630.82</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>SHBL</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="n">
+        <v>14077.5</v>
+      </c>
+      <c r="C123" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D123" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E123" s="5" t="n">
+        <v>14201.45</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>SHIVM</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="n">
+        <v>75586.92999999999</v>
+      </c>
+      <c r="C124" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D124" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E124" s="5" t="n">
+        <v>81318.45</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>SHLB</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="n">
+        <v>88948.92999999999</v>
+      </c>
+      <c r="C125" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D125" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E125" s="5" t="n">
+        <v>111121.36</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="inlineStr">
+        <is>
+          <t>SICL</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="n">
+        <v>35858.88</v>
+      </c>
+      <c r="C126" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D126" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E126" s="5" t="n">
+        <v>42813.75</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>SIFC</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="n">
+        <v>4742.62</v>
+      </c>
+      <c r="C127" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D127" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E127" s="5" t="n">
+        <v>7595.32</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>SIGS2</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="n">
+        <v>238.2</v>
+      </c>
+      <c r="C128" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D128" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="E128" s="5" t="n">
+        <v>270.89</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>SINDU</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="n">
+        <v>28495.17</v>
+      </c>
+      <c r="C129" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D129" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="E129" s="5" t="n">
+        <v>42235.73</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="4" t="inlineStr">
+        <is>
+          <t>SKBBL</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="n">
+        <v>19306.03</v>
+      </c>
+      <c r="C130" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D130" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E130" s="5" t="n">
+        <v>21663.36</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>SLBBL</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="n">
+        <v>71040.12</v>
+      </c>
+      <c r="C131" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D131" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E131" s="5" t="n">
+        <v>75620.08</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>SLBSL</t>
+        </is>
+      </c>
+      <c r="B132" s="5" t="n">
+        <v>50725.23</v>
+      </c>
+      <c r="C132" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D132" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E132" s="5" t="n">
+        <v>88392</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>SLCF</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="n">
+        <v>1496.9</v>
+      </c>
+      <c r="C133" s="6" t="n">
+        <v>141</v>
+      </c>
+      <c r="D133" s="6" t="n">
+        <v>141</v>
+      </c>
+      <c r="E133" s="5" t="n">
+        <v>1617.11</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>SMATA</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="n">
+        <v>16767.55</v>
+      </c>
+      <c r="C134" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D134" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E134" s="5" t="n">
+        <v>17509</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>SMB</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="n">
+        <v>153518.07</v>
+      </c>
+      <c r="C135" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D135" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E135" s="5" t="n">
+        <v>200430.1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="4" t="inlineStr">
+        <is>
+          <t>SMFBS</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="n">
+        <v>43261.44</v>
+      </c>
+      <c r="C136" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D136" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E136" s="5" t="n">
+        <v>47351.58</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>SMHL</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="n">
+        <v>30172.54</v>
+      </c>
+      <c r="C137" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D137" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E137" s="5" t="n">
+        <v>32965.72</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>SPC</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="n">
+        <v>7488.88</v>
+      </c>
+      <c r="C138" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="D138" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E138" s="5" t="n">
+        <v>9224.18</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>STC</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="n">
+        <v>318594.79</v>
+      </c>
+      <c r="C139" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D139" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E139" s="5" t="n">
+        <v>331476.81</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>SWASTIK</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="n">
+        <v>136027.72</v>
+      </c>
+      <c r="C140" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D140" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E140" s="5" t="n">
+        <v>162766.85</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>SWMF</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="n">
+        <v>9881.83</v>
+      </c>
+      <c r="C141" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D141" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E141" s="5" t="n">
+        <v>11481.69</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="4" t="inlineStr">
+        <is>
+          <t>SYPNL</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="n">
+        <v>81399.73</v>
+      </c>
+      <c r="C142" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D142" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E142" s="5" t="n">
+        <v>84659.96000000001</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>TRH</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="n">
+        <v>14596.35</v>
+      </c>
+      <c r="C143" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="D143" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E143" s="5" t="n">
+        <v>52418.31</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="4" t="inlineStr">
+        <is>
+          <t>TTL</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="n">
+        <v>71306.03999999999</v>
+      </c>
+      <c r="C144" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="D144" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="E144" s="5" t="n">
+        <v>77612.23</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>TVCL</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="n">
+        <v>49595.22</v>
+      </c>
+      <c r="C145" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="D145" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="E145" s="5" t="n">
+        <v>53078.74</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="4" t="inlineStr">
+        <is>
+          <t>ULBSL</t>
+        </is>
+      </c>
+      <c r="B146" s="5" t="n">
+        <v>757756.79</v>
+      </c>
+      <c r="C146" s="6" t="n">
+        <v>190</v>
+      </c>
+      <c r="D146" s="6" t="n">
+        <v>190</v>
+      </c>
+      <c r="E146" s="5" t="n">
+        <v>1145700.65</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>UMHL</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="n">
+        <v>28684.37</v>
+      </c>
+      <c r="C147" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="D147" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="E147" s="5" t="n">
+        <v>31408.5</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="4" t="inlineStr">
+        <is>
+          <t>UMRH</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="n">
+        <v>61703.88</v>
+      </c>
+      <c r="C148" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="D148" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="E148" s="5" t="n">
+        <v>85610.08</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>UNL</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="n">
+        <v>3625945.75</v>
+      </c>
+      <c r="C149" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="D149" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="E149" s="5" t="n">
+        <v>4072220.95</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="4" t="inlineStr">
+        <is>
+          <t>USHL</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="n">
+        <v>57063.44</v>
+      </c>
+      <c r="C150" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="D150" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="E150" s="5" t="n">
+        <v>69379.27</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>USLB</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="n">
+        <v>23622.46</v>
+      </c>
+      <c r="C151" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D151" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E151" s="5" t="n">
+        <v>26384.49</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="4" t="inlineStr">
+        <is>
+          <t>WNLB</t>
+        </is>
+      </c>
+      <c r="B152" s="5" t="n">
+        <v>211443.3</v>
+      </c>
+      <c r="C152" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="D152" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="E152" s="5" t="n">
+        <v>292652.78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>